<commit_message>
sync README with simplified xlsx evaluation table (28 -> 21 items)
- Remove threshold management section (old items 11-17)
- Renumber all items to match xlsx: error prevention 11-16, emergency 17-19, logging 20-21
- Update task descriptions and scoring criteria accordingly
</commit_message>
<xml_diff>
--- a/docs/期货程序化交易系统功能标准符合性评估表.xlsx
+++ b/docs/期货程序化交易系统功能标准符合性评估表.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowHeight="18375" activeTab="2"/>
+    <workbookView windowWidth="27945" windowHeight="11925" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="提测须知" sheetId="3" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="97">
   <si>
     <t>修订历史</t>
   </si>
@@ -279,32 +279,6 @@
   </si>
   <si>
     <t>是否能正常监测单合约重复撤单交易指令数量</t>
-  </si>
-  <si>
-    <t>是否提供报单笔数的阈值设置功能</t>
-  </si>
-  <si>
-    <t>检查期货程序化交易系统是否能够设置报单笔数、撤单笔数、重复报单笔数等指标阈值；设置指标阈值后，使用期货程序化交易系统进行交易，
-当监测指标达到或超过设置阈值时，检查期货程序化交易系统是否能够通过一种或多种方式进行预警，
-预警方式包括但不限于弹窗提示、声音提示、短信或邮件通知</t>
-  </si>
-  <si>
-    <t>验证开仓单报单笔数等于或大于设置的阈值时，是否能够通过一种或多种方式进行预警，预警方式包括但不限于弹窗提示、声音提示、短信或邮件通知</t>
-  </si>
-  <si>
-    <t>验证重复开仓单报单笔数等于或大于设置的阈值时，是否能够通过一种或多种方式进行预警，预警方式包括但不限于弹窗提示、声音提示、短信或邮件通知</t>
-  </si>
-  <si>
-    <t>验证平仓单报单笔数等于或大于设置的阈值时，是否能够通过一种或多种方式进行预警，预警方式包括但不限于弹窗提示、声音提示、短信或邮件通知</t>
-  </si>
-  <si>
-    <t>验证重复平仓单报单笔数等于或大于设置的阈值时，是否能够通过一种或多种方式进行预警，预警方式包括但不限于弹窗提示、声音提示、短信或邮件通知</t>
-  </si>
-  <si>
-    <t>验证撤单笔数等于或大于设置的阈值时，是否能够通过一种或多种方式进行预警，预警方式包括但不限于弹窗提示、声音提示、短信或邮件通知</t>
-  </si>
-  <si>
-    <t>验证重复撤单报单笔数等于或大于设置的阈值时，是否能够通过一种或多种方式进行预警，预警方式包括但不限于弹窗提示、声音提示、短信或邮件通知</t>
   </si>
   <si>
     <t>当合约代码错误时，系统是否能检查出合约代码错误</t>
@@ -1290,24 +1264,33 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1320,21 +1303,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1361,9 +1338,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
@@ -1694,13 +1668,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>601980</xdr:colOff>
-      <xdr:row>32</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>15240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>281940</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>99060</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
@@ -1710,7 +1684,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="601980" y="10213340"/>
+          <a:off x="601980" y="6708140"/>
           <a:ext cx="8544560" cy="1893570"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2068,7 +2042,7 @@
     <col min="4" max="4" width="27.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:16">
       <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
@@ -2076,7 +2050,7 @@
       <c r="C1" s="39"/>
       <c r="D1" s="39"/>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:16">
       <c r="A2" s="39" t="s">
         <v>1</v>
       </c>
@@ -2344,7 +2318,7 @@
       <c r="O13" s="40"/>
       <c r="P13" s="40"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:16">
       <c r="A14" s="51" t="s">
         <v>28</v>
       </c>
@@ -2358,7 +2332,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:16">
       <c r="A15" s="51"/>
       <c r="B15" s="51" t="s">
         <v>30</v>
@@ -2370,7 +2344,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:16">
       <c r="A16" s="51" t="s">
         <v>31</v>
       </c>
@@ -2454,39 +2428,39 @@
       <c r="F1" s="27"/>
       <c r="G1" s="27"/>
       <c r="H1" s="27"/>
-      <c r="I1" s="37"/>
+      <c r="I1" s="28"/>
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:9">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="30" t="s">
+      <c r="B2" s="30"/>
+      <c r="C2" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="30" t="s">
+      <c r="D2" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="30" t="s">
+      <c r="E2" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="28" t="s">
+      <c r="F2" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="G2" s="29"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:9">
-      <c r="A3" s="28"/>
-      <c r="B3" s="29"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
+      <c r="A3" s="29"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
     </row>
     <row r="4" ht="43" customHeight="1" spans="1:9">
       <c r="A4" s="26" t="s">
@@ -2499,61 +2473,61 @@
       <c r="F4" s="27"/>
       <c r="G4" s="27"/>
       <c r="H4" s="27"/>
-      <c r="I4" s="37"/>
+      <c r="I4" s="28"/>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:9">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="C5" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="32" t="s">
+      <c r="E5" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="32" t="s">
+      <c r="F5" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="32" t="s">
+      <c r="G5" s="33" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="32" t="s">
+      <c r="H5" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="I5" s="32" t="s">
+      <c r="I5" s="33" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:9">
-      <c r="A6" s="34"/>
-      <c r="B6" s="35"/>
-      <c r="C6" s="36" t="s">
+      <c r="A6" s="35"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="34"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="32"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="33"/>
       <c r="I6" s="38"/>
     </row>
     <row r="7" customFormat="1" ht="34" customHeight="1" spans="1:9">
-      <c r="A7" s="34"/>
-      <c r="B7" s="35"/>
-      <c r="C7" s="36" t="s">
+      <c r="A7" s="35"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="34"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="34"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="32"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="35"/>
+      <c r="G7" s="35"/>
+      <c r="H7" s="33"/>
       <c r="I7" s="38"/>
     </row>
   </sheetData>
@@ -2585,7 +2559,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="B1:I30"/>
+  <dimension ref="B1:I23"/>
   <sheetFormatPr defaultColWidth="8.89166666666667" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="8.89166666666667" style="1" customWidth="1"/>
@@ -2600,7 +2574,7 @@
     <col min="10" max="16384" width="58.775" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="29" customHeight="1" spans="2:8">
+    <row r="1" ht="29" customHeight="1" spans="2:9">
       <c r="B1" s="3" t="s">
         <v>53</v>
       </c>
@@ -2655,16 +2629,16 @@
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
-      <c r="I3" s="23" t="s">
+      <c r="I3" s="13" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="4" ht="15" spans="2:9">
-      <c r="B4" s="13">
+      <c r="B4" s="14">
         <v>2</v>
       </c>
       <c r="C4" s="9"/>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="15" t="s">
         <v>19</v>
       </c>
       <c r="E4" s="10" t="s">
@@ -2675,16 +2649,16 @@
       </c>
       <c r="G4" s="12"/>
       <c r="H4" s="11"/>
-      <c r="I4" s="24" t="s">
+      <c r="I4" s="16" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="5" ht="15" spans="2:9">
-      <c r="B5" s="15">
+      <c r="B5" s="17">
         <v>3</v>
       </c>
       <c r="C5" s="9"/>
-      <c r="D5" s="14"/>
+      <c r="D5" s="15"/>
       <c r="E5" s="10" t="s">
         <v>68</v>
       </c>
@@ -2693,14 +2667,14 @@
       </c>
       <c r="G5" s="12"/>
       <c r="H5" s="11"/>
-      <c r="I5" s="24"/>
+      <c r="I5" s="16"/>
     </row>
     <row r="6" ht="15" spans="2:9">
-      <c r="B6" s="15">
+      <c r="B6" s="17">
         <v>4</v>
       </c>
       <c r="C6" s="9"/>
-      <c r="D6" s="14"/>
+      <c r="D6" s="15"/>
       <c r="E6" s="10" t="s">
         <v>69</v>
       </c>
@@ -2709,19 +2683,19 @@
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="11"/>
-      <c r="I6" s="17"/>
+      <c r="I6" s="18"/>
     </row>
     <row r="7" ht="36" customHeight="1" spans="2:9">
       <c r="B7" s="8">
         <v>5</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="18" t="s">
         <v>71</v>
       </c>
       <c r="F7" s="11" t="s">
@@ -2729,16 +2703,16 @@
       </c>
       <c r="G7" s="12"/>
       <c r="H7" s="12"/>
-      <c r="I7" s="17" t="s">
+      <c r="I7" s="18" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="8" ht="15" spans="2:9">
-      <c r="B8" s="13">
+      <c r="B8" s="14">
         <v>6</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="14" t="s">
+      <c r="C8" s="19"/>
+      <c r="D8" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="10" t="s">
@@ -2749,16 +2723,16 @@
       </c>
       <c r="G8" s="12"/>
       <c r="H8" s="11"/>
-      <c r="I8" s="24" t="s">
+      <c r="I8" s="16" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="9" ht="15" spans="2:9">
-      <c r="B9" s="15">
+      <c r="B9" s="17">
         <v>7</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="18"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="20"/>
       <c r="E9" s="10" t="s">
         <v>75</v>
       </c>
@@ -2767,14 +2741,14 @@
       </c>
       <c r="G9" s="12"/>
       <c r="H9" s="12"/>
-      <c r="I9" s="17"/>
+      <c r="I9" s="18"/>
     </row>
     <row r="10" ht="15" spans="2:9">
-      <c r="B10" s="15">
+      <c r="B10" s="17">
         <v>8</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="14" t="s">
+      <c r="C10" s="19"/>
+      <c r="D10" s="15" t="s">
         <v>23</v>
       </c>
       <c r="E10" s="10" t="s">
@@ -2785,7 +2759,7 @@
       </c>
       <c r="G10" s="12"/>
       <c r="H10" s="11"/>
-      <c r="I10" s="24" t="s">
+      <c r="I10" s="16" t="s">
         <v>78</v>
       </c>
     </row>
@@ -2793,8 +2767,8 @@
       <c r="B11" s="8">
         <v>9</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="20"/>
       <c r="E11" s="10" t="s">
         <v>79</v>
       </c>
@@ -2803,14 +2777,14 @@
       </c>
       <c r="G11" s="12"/>
       <c r="H11" s="11"/>
-      <c r="I11" s="24"/>
+      <c r="I11" s="16"/>
     </row>
     <row r="12" ht="15" spans="2:9">
-      <c r="B12" s="13">
+      <c r="B12" s="14">
         <v>10</v>
       </c>
-      <c r="C12" s="16"/>
-      <c r="D12" s="18"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="20"/>
       <c r="E12" s="10" t="s">
         <v>80</v>
       </c>
@@ -2819,17 +2793,17 @@
       </c>
       <c r="G12" s="12"/>
       <c r="H12" s="12"/>
-      <c r="I12" s="17"/>
+      <c r="I12" s="18"/>
     </row>
     <row r="13" ht="15" spans="2:9">
-      <c r="B13" s="15">
+      <c r="B13" s="17">
         <v>11</v>
       </c>
-      <c r="C13" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>27</v>
+      <c r="C13" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>81</v>
@@ -2839,16 +2813,16 @@
       </c>
       <c r="G13" s="12"/>
       <c r="H13" s="12"/>
-      <c r="I13" s="24" t="s">
+      <c r="I13" s="16" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="14" ht="43.5" spans="2:9">
+    <row r="14" ht="29.25" spans="2:9">
       <c r="B14" s="8">
         <v>12</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="14"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="15"/>
       <c r="E14" s="10" t="s">
         <v>83</v>
       </c>
@@ -2857,26 +2831,32 @@
       </c>
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
-      <c r="I14" s="25"/>
-    </row>
-    <row r="15" ht="43.5" spans="2:9">
-      <c r="B15" s="13"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="14"/>
+      <c r="I14" s="21"/>
+    </row>
+    <row r="15" ht="29.25" spans="2:9">
+      <c r="B15" s="8">
+        <v>13</v>
+      </c>
+      <c r="C15" s="19"/>
+      <c r="D15" s="15"/>
       <c r="E15" s="10" t="s">
         <v>84</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="25"/>
-    </row>
-    <row r="16" ht="43.5" spans="2:9">
-      <c r="B16" s="13"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="14"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="13"/>
+    </row>
+    <row r="16" ht="29.25" spans="2:9">
+      <c r="B16" s="14">
+        <v>14</v>
+      </c>
+      <c r="C16" s="19"/>
+      <c r="D16" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="E16" s="10" t="s">
         <v>85</v>
       </c>
@@ -2885,282 +2865,163 @@
       </c>
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
-      <c r="I16" s="25"/>
-    </row>
-    <row r="17" ht="43.5" spans="2:9">
-      <c r="B17" s="13"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="14"/>
+      <c r="I16" s="21" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" ht="29.25" spans="2:9">
+      <c r="B17" s="17">
+        <v>15</v>
+      </c>
+      <c r="C17" s="19"/>
+      <c r="D17" s="15"/>
       <c r="E17" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
-      <c r="I17" s="25"/>
-    </row>
-    <row r="18" ht="43.5" spans="2:9">
-      <c r="B18" s="13"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="14"/>
+      <c r="I17" s="21"/>
+    </row>
+    <row r="18" ht="29.25" spans="2:9">
+      <c r="B18" s="8">
+        <v>16</v>
+      </c>
+      <c r="C18" s="19"/>
+      <c r="D18" s="15"/>
       <c r="E18" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F18" s="11" t="s">
         <v>64</v>
       </c>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
-      <c r="I18" s="25"/>
-    </row>
-    <row r="19" ht="43.5" spans="2:9">
-      <c r="B19" s="13">
+      <c r="I18" s="13"/>
+    </row>
+    <row r="19" ht="34" customHeight="1" spans="2:9">
+      <c r="B19" s="8">
         <v>17</v>
       </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="14"/>
+      <c r="C19" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>32</v>
+      </c>
       <c r="E19" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F19" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="18" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" ht="15" spans="2:9">
+      <c r="B20" s="14">
+        <v>18</v>
+      </c>
+      <c r="C20" s="22"/>
+      <c r="D20" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F20" s="11" t="s">
         <v>77</v>
-      </c>
-      <c r="G19" s="12"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="23"/>
-    </row>
-    <row r="20" ht="15" spans="2:9">
-      <c r="B20" s="15">
-        <v>18</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>64</v>
       </c>
       <c r="G20" s="12"/>
       <c r="H20" s="12"/>
-      <c r="I20" s="24" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="21" ht="29.25" spans="2:9">
-      <c r="B21" s="8">
+      <c r="I20" s="21" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" ht="15" spans="2:9">
+      <c r="B21" s="17">
         <v>19</v>
       </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="14"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="11"/>
       <c r="E21" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>
-      <c r="I21" s="25"/>
-    </row>
-    <row r="22" ht="29.25" spans="2:9">
+      <c r="I21" s="13"/>
+    </row>
+    <row r="22" ht="15" spans="2:9">
       <c r="B22" s="8">
         <v>20</v>
       </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="10" t="s">
-        <v>92</v>
+      <c r="C22" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>94</v>
       </c>
       <c r="F22" s="11" t="s">
         <v>64</v>
       </c>
       <c r="G22" s="12"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="23"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="16" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="23" ht="29.25" spans="2:9">
-      <c r="B23" s="13">
+      <c r="B23" s="14">
         <v>21</v>
       </c>
-      <c r="C23" s="16"/>
-      <c r="D23" s="14" t="s">
-        <v>30</v>
-      </c>
+      <c r="C23" s="24"/>
+      <c r="D23" s="11"/>
       <c r="E23" s="10" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="F23" s="11" t="s">
         <v>64</v>
       </c>
       <c r="G23" s="12"/>
-      <c r="H23" s="12"/>
-      <c r="I23" s="25" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="24" ht="29.25" spans="2:9">
-      <c r="B24" s="15">
-        <v>22</v>
-      </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="G24" s="12"/>
-      <c r="H24" s="12"/>
-      <c r="I24" s="25"/>
-    </row>
-    <row r="25" ht="29.25" spans="2:9">
-      <c r="B25" s="8">
-        <v>23</v>
-      </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="F25" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="23"/>
-    </row>
-    <row r="26" ht="34" customHeight="1" spans="2:9">
-      <c r="B26" s="8">
-        <v>24</v>
-      </c>
-      <c r="C26" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="D26" s="20" t="s">
-        <v>32</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="F26" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
-      <c r="I26" s="17" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="27" ht="15" spans="2:9">
-      <c r="B27" s="13">
-        <v>25</v>
-      </c>
-      <c r="C27" s="19"/>
-      <c r="D27" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="F27" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="G27" s="12"/>
-      <c r="H27" s="12"/>
-      <c r="I27" s="25" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="28" ht="15" spans="2:9">
-      <c r="B28" s="15">
-        <v>26</v>
-      </c>
-      <c r="C28" s="19"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="F28" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="G28" s="12"/>
-      <c r="H28" s="12"/>
-      <c r="I28" s="23"/>
-    </row>
-    <row r="29" ht="15" spans="2:9">
-      <c r="B29" s="8">
-        <v>27</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="D29" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="E29" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="F29" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
-      <c r="I29" s="24" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="30" ht="29.25" spans="2:9">
-      <c r="B30" s="13">
-        <v>28</v>
-      </c>
-      <c r="C30" s="21"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="F30" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="G30" s="12"/>
-      <c r="H30" s="22"/>
-      <c r="I30" s="23"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="20">
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="C3:C6"/>
     <mergeCell ref="C7:C12"/>
-    <mergeCell ref="C13:C19"/>
-    <mergeCell ref="C20:C25"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="C13:C18"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="C22:C23"/>
     <mergeCell ref="D4:D6"/>
     <mergeCell ref="D8:D9"/>
     <mergeCell ref="D10:D12"/>
-    <mergeCell ref="D13:D19"/>
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="D23:D25"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="D16:D18"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="D22:D23"/>
     <mergeCell ref="I4:I6"/>
     <mergeCell ref="I8:I9"/>
     <mergeCell ref="I10:I12"/>
-    <mergeCell ref="I13:I19"/>
-    <mergeCell ref="I20:I22"/>
-    <mergeCell ref="I23:I25"/>
-    <mergeCell ref="I27:I28"/>
-    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="I13:I15"/>
+    <mergeCell ref="I16:I18"/>
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="I22:I23"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G30">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G12 G13:G23">
       <formula1>"是,否"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>